<commit_message>
task 2 "to be revised"
</commit_message>
<xml_diff>
--- a/Lab03 - Data Acquisition/notebooks/task2_deliverables/task3_results.xlsx
+++ b/Lab03 - Data Acquisition/notebooks/task2_deliverables/task3_results.xlsx
@@ -79,22 +79,22 @@
     <t>2014-02-25T08:00:08Z</t>
   </si>
   <si>
-    <t>2026-03-02T12:43:15Z</t>
-  </si>
-  <si>
-    <t>2026-03-02T12:26:45Z</t>
-  </si>
-  <si>
-    <t>2026-03-02T12:00:55Z</t>
-  </si>
-  <si>
-    <t>2026-03-02T09:05:10Z</t>
-  </si>
-  <si>
-    <t>2026-03-02T06:32:43Z</t>
-  </si>
-  <si>
-    <t>Exported at: 2026-03-02 14:50:04.238151</t>
+    <t>2026-03-05T22:34:46Z</t>
+  </si>
+  <si>
+    <t>2026-03-05T22:36:30Z</t>
+  </si>
+  <si>
+    <t>2026-03-05T21:44:37Z</t>
+  </si>
+  <si>
+    <t>2026-03-05T17:52:10Z</t>
+  </si>
+  <si>
+    <t>2026-03-05T21:23:08Z</t>
+  </si>
+  <si>
+    <t>Exported at: 2026-03-06 00:44:54.386230</t>
   </si>
 </sst>
 </file>
@@ -479,16 +479,16 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>193960</v>
+        <v>194010</v>
       </c>
       <c r="C2">
-        <v>75215</v>
+        <v>75217</v>
       </c>
       <c r="D2">
-        <v>3594</v>
+        <v>3599</v>
       </c>
       <c r="E2">
-        <v>193960</v>
+        <v>194010</v>
       </c>
       <c r="F2" t="s">
         <v>13</v>
@@ -505,16 +505,16 @@
         <v>9</v>
       </c>
       <c r="B3">
-        <v>97880</v>
+        <v>97984</v>
       </c>
       <c r="C3">
-        <v>27034</v>
+        <v>27081</v>
       </c>
       <c r="D3">
-        <v>18060</v>
+        <v>18086</v>
       </c>
       <c r="E3">
-        <v>97880</v>
+        <v>97984</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -531,16 +531,16 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>65267</v>
+        <v>65297</v>
       </c>
       <c r="C4">
-        <v>26737</v>
+        <v>26751</v>
       </c>
       <c r="D4">
-        <v>2147</v>
+        <v>2136</v>
       </c>
       <c r="E4">
-        <v>65267</v>
+        <v>65297</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -557,16 +557,16 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>63887</v>
+        <v>63911</v>
       </c>
       <c r="C5">
-        <v>19713</v>
+        <v>19714</v>
       </c>
       <c r="D5">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="E5">
-        <v>63887</v>
+        <v>63911</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>
@@ -583,16 +583,16 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>42909</v>
+        <v>42931</v>
       </c>
       <c r="C6">
-        <v>29083</v>
+        <v>29089</v>
       </c>
       <c r="D6">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E6">
-        <v>42909</v>
+        <v>42931</v>
       </c>
       <c r="F6" t="s">
         <v>15</v>

</xml_diff>